<commit_message>
Refactor and expand instrument solution mappings in `instruments_tree.json`.
Reorganized entries for better structure and accuracy, swapped inconsistent key placements, and standardized solution mappings for newly added and updated instruments. Simplified naming conventions and introduced missing configurations such as "Q-Exactive HF-X" and "GC Orbitrap Q-Exactive".
</commit_message>
<xml_diff>
--- a/Instrument_tree.xlsx
+++ b/Instrument_tree.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Axel\PYTHON\FragHub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6349F7A3-53C4-4350-AF5D-171651E5F29B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AAF4291-818D-48B7-BAEF-D188AD6F7DB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AB SCIEX" sheetId="1" r:id="rId1"/>
@@ -37,12 +37,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1854" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1866" uniqueCount="323">
   <si>
     <t>MARQUES</t>
   </si>
@@ -1008,6 +1011,9 @@
   </si>
   <si>
     <t>EB</t>
+  </si>
+  <si>
+    <t>Excedion Pro</t>
   </si>
 </sst>
 </file>
@@ -3598,7 +3604,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
@@ -4633,10 +4639,48 @@
       <c r="G51" s="3"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B52" s="3"/>
+      <c r="A52" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D52" t="s">
+        <v>52</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D53" t="s">
+        <v>52</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>